<commit_message>
Refactor OAH indicators and observations
</commit_message>
<xml_diff>
--- a/_samples/heathIndicator-OAH.xlsx
+++ b/_samples/heathIndicator-OAH.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29711"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universidadedecoimbra154.sharepoint.com/sites/OneAquaHealth/Documentos Partilhados/OneAquaHealth Teams/ONEAQUAHEALTH shared/WP3_Human health indicators, behaviours and policies/T3.1 INDICATORS/Research Sites data for OAH/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\oah\_samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B4E6F6B-9127-49C1-9343-317EE0A9C8BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84C9302-11E3-4128-842E-2D6739299DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27480" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="759" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-6510" yWindow="-21710" windowWidth="38620" windowHeight="21100" tabRatio="759" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BN_Legenda" sheetId="26" r:id="rId1"/>
@@ -2093,6 +2093,12 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="18" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2111,11 +2117,14 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -2124,15 +2133,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2256,6 +2256,16 @@
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3042,16 +3052,6 @@
         </patternFill>
       </fill>
       <alignment vertical="center" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0"/>
@@ -5817,27 +5817,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{35049DD6-056E-E549-A047-2F0D62E276A7}" name="filtered_dataset3423" displayName="filtered_dataset3423" ref="A1:S2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{35049DD6-056E-E549-A047-2F0D62E276A7}" name="filtered_dataset3423" displayName="filtered_dataset3423" ref="A1:S2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <tableColumns count="19">
-    <tableColumn id="2" xr3:uid="{E785F718-750B-7F4C-A940-18B6C08AE3D9}" name="Colonna1" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{67C25394-600C-BD4D-B2DF-128C072102D8}" name="BN1" dataDxfId="33" dataCellStyle="Normale 2"/>
-    <tableColumn id="4" xr3:uid="{8F121421-8207-B640-A2DF-2152A7F5792F}" name="BN2" dataDxfId="32" dataCellStyle="Normale 2"/>
-    <tableColumn id="5" xr3:uid="{FC29E100-ED34-D543-A112-469C7AA3196E}" name="BN3" dataDxfId="31" dataCellStyle="Normale 2"/>
-    <tableColumn id="6" xr3:uid="{35251F84-836F-5545-AF20-CD4BDEBA3A8C}" name="BN4+BN13" dataDxfId="30" dataCellStyle="Normale 2"/>
-    <tableColumn id="7" xr3:uid="{0E2581ED-5EC2-B344-B50E-3BAC2FC46BFF}" name="BN5" dataDxfId="29" dataCellStyle="Normale 2"/>
-    <tableColumn id="8" xr3:uid="{0691BD33-1714-594D-BF6D-F601D40AF88F}" name="BN6" dataDxfId="28" dataCellStyle="Normale 2"/>
-    <tableColumn id="9" xr3:uid="{997BB5E6-58A9-E64C-8F5A-858CCA787EBA}" name="BN7" dataDxfId="27" dataCellStyle="Normale 2"/>
-    <tableColumn id="10" xr3:uid="{BA976491-A323-8149-BB30-2389869B43C2}" name="BN8" dataDxfId="26" dataCellStyle="Normale 2"/>
-    <tableColumn id="11" xr3:uid="{B6F191CB-1511-7A43-B9ED-CA9AE69C962C}" name="BN9" dataDxfId="25" dataCellStyle="Normale 2"/>
-    <tableColumn id="12" xr3:uid="{8529D515-5DED-9045-BBA5-8C97A315EF1F}" name="BN10" dataDxfId="24" dataCellStyle="Normale 2"/>
-    <tableColumn id="13" xr3:uid="{66ED7FB9-E93D-A549-BC6C-9B23DE9FB4F3}" name="BN11" dataDxfId="23" dataCellStyle="Normale 2"/>
-    <tableColumn id="14" xr3:uid="{E13F466E-403D-B643-A13B-A9E3F9059BEC}" name="BN12" dataDxfId="22" dataCellStyle="Normale 2"/>
-    <tableColumn id="16" xr3:uid="{B17D3634-CC60-1B4D-A4FC-C9A217637ACC}" name="BN14" dataDxfId="21" dataCellStyle="Normale 2"/>
-    <tableColumn id="17" xr3:uid="{7A993824-F979-3047-8684-63805BBACB9C}" name="BN15+BN16" dataDxfId="20" dataCellStyle="Normale 2"/>
-    <tableColumn id="19" xr3:uid="{8CFEB265-412B-1041-858A-B4DA316F1C0E}" name="BN17" dataDxfId="19" dataCellStyle="Normale 2"/>
-    <tableColumn id="20" xr3:uid="{22D85DC7-6E9A-CE4E-B7D4-1C0C3D57F5D1}" name="BN18" dataDxfId="18" dataCellStyle="Normale 2"/>
-    <tableColumn id="21" xr3:uid="{24656BD6-6D25-3C4E-AB8D-1DB7589E7B97}" name="BN19" dataDxfId="17" dataCellStyle="Normale 2"/>
-    <tableColumn id="22" xr3:uid="{4ACC59A5-CF52-694B-81DC-44DECA00FE46}" name="BN20" dataDxfId="16" dataCellStyle="Normale 2"/>
+    <tableColumn id="2" xr3:uid="{E785F718-750B-7F4C-A940-18B6C08AE3D9}" name="Colonna1" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{67C25394-600C-BD4D-B2DF-128C072102D8}" name="BN1" dataDxfId="34" dataCellStyle="Normale 2"/>
+    <tableColumn id="4" xr3:uid="{8F121421-8207-B640-A2DF-2152A7F5792F}" name="BN2" dataDxfId="33" dataCellStyle="Normale 2"/>
+    <tableColumn id="5" xr3:uid="{FC29E100-ED34-D543-A112-469C7AA3196E}" name="BN3" dataDxfId="32" dataCellStyle="Normale 2"/>
+    <tableColumn id="6" xr3:uid="{35251F84-836F-5545-AF20-CD4BDEBA3A8C}" name="BN4+BN13" dataDxfId="31" dataCellStyle="Normale 2"/>
+    <tableColumn id="7" xr3:uid="{0E2581ED-5EC2-B344-B50E-3BAC2FC46BFF}" name="BN5" dataDxfId="30" dataCellStyle="Normale 2"/>
+    <tableColumn id="8" xr3:uid="{0691BD33-1714-594D-BF6D-F601D40AF88F}" name="BN6" dataDxfId="29" dataCellStyle="Normale 2"/>
+    <tableColumn id="9" xr3:uid="{997BB5E6-58A9-E64C-8F5A-858CCA787EBA}" name="BN7" dataDxfId="28" dataCellStyle="Normale 2"/>
+    <tableColumn id="10" xr3:uid="{BA976491-A323-8149-BB30-2389869B43C2}" name="BN8" dataDxfId="27" dataCellStyle="Normale 2"/>
+    <tableColumn id="11" xr3:uid="{B6F191CB-1511-7A43-B9ED-CA9AE69C962C}" name="BN9" dataDxfId="26" dataCellStyle="Normale 2"/>
+    <tableColumn id="12" xr3:uid="{8529D515-5DED-9045-BBA5-8C97A315EF1F}" name="BN10" dataDxfId="25" dataCellStyle="Normale 2"/>
+    <tableColumn id="13" xr3:uid="{66ED7FB9-E93D-A549-BC6C-9B23DE9FB4F3}" name="BN11" dataDxfId="24" dataCellStyle="Normale 2"/>
+    <tableColumn id="14" xr3:uid="{E13F466E-403D-B643-A13B-A9E3F9059BEC}" name="BN12" dataDxfId="23" dataCellStyle="Normale 2"/>
+    <tableColumn id="16" xr3:uid="{B17D3634-CC60-1B4D-A4FC-C9A217637ACC}" name="BN14" dataDxfId="22" dataCellStyle="Normale 2"/>
+    <tableColumn id="17" xr3:uid="{7A993824-F979-3047-8684-63805BBACB9C}" name="BN15+BN16" dataDxfId="21" dataCellStyle="Normale 2"/>
+    <tableColumn id="19" xr3:uid="{8CFEB265-412B-1041-858A-B4DA316F1C0E}" name="BN17" dataDxfId="20" dataCellStyle="Normale 2"/>
+    <tableColumn id="20" xr3:uid="{22D85DC7-6E9A-CE4E-B7D4-1C0C3D57F5D1}" name="BN18" dataDxfId="19" dataCellStyle="Normale 2"/>
+    <tableColumn id="21" xr3:uid="{24656BD6-6D25-3C4E-AB8D-1DB7589E7B97}" name="BN19" dataDxfId="18" dataCellStyle="Normale 2"/>
+    <tableColumn id="22" xr3:uid="{4ACC59A5-CF52-694B-81DC-44DECA00FE46}" name="BN20" dataDxfId="17" dataCellStyle="Normale 2"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6886,11 +6886,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5655DEA0-8796-F74B-B1B2-985E15B7C23E}">
   <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="14" style="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" style="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.85546875" style="36"/>
+    <col min="2" max="2" width="16.3984375" style="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.86328125" style="36"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7072,11 +7072,11 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:S17"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="82.28515625" style="116" customWidth="1"/>
-    <col min="2" max="19" width="8.85546875" style="116" customWidth="1"/>
-    <col min="20" max="16384" width="10.85546875" style="116"/>
+    <col min="1" max="1" width="82.265625" style="116" customWidth="1"/>
+    <col min="2" max="19" width="8.86328125" style="116" customWidth="1"/>
+    <col min="20" max="16384" width="10.86328125" style="116"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="198" customHeight="1">
@@ -7139,38 +7139,38 @@
       <c r="C2" s="125" t="s">
         <v>280</v>
       </c>
-      <c r="D2" s="161" t="s">
+      <c r="D2" s="159" t="s">
         <v>236</v>
       </c>
-      <c r="E2" s="162"/>
-      <c r="F2" s="161" t="s">
+      <c r="E2" s="160"/>
+      <c r="F2" s="159" t="s">
         <v>238</v>
       </c>
-      <c r="G2" s="162"/>
-      <c r="H2" s="161" t="s">
+      <c r="G2" s="160"/>
+      <c r="H2" s="159" t="s">
         <v>241</v>
       </c>
-      <c r="I2" s="162"/>
-      <c r="J2" s="161" t="s">
+      <c r="I2" s="160"/>
+      <c r="J2" s="159" t="s">
         <v>244</v>
       </c>
-      <c r="K2" s="162"/>
-      <c r="L2" s="161" t="s">
+      <c r="K2" s="160"/>
+      <c r="L2" s="159" t="s">
         <v>253</v>
       </c>
-      <c r="M2" s="162"/>
-      <c r="N2" s="161" t="s">
+      <c r="M2" s="160"/>
+      <c r="N2" s="159" t="s">
         <v>256</v>
       </c>
-      <c r="O2" s="162"/>
-      <c r="P2" s="161" t="s">
+      <c r="O2" s="160"/>
+      <c r="P2" s="159" t="s">
         <v>258</v>
       </c>
-      <c r="Q2" s="162"/>
-      <c r="R2" s="158" t="s">
+      <c r="Q2" s="160"/>
+      <c r="R2" s="161" t="s">
         <v>261</v>
       </c>
-      <c r="S2" s="158"/>
+      <c r="S2" s="161"/>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="126" t="s">
@@ -7622,51 +7622,51 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="17.100000000000001">
+    <row r="11" spans="1:19">
       <c r="A11" s="116" t="s">
         <v>287</v>
       </c>
-      <c r="D11" s="159">
+      <c r="D11" s="162">
         <v>0.08</v>
       </c>
-      <c r="E11" s="160"/>
-      <c r="F11" s="159">
+      <c r="E11" s="163"/>
+      <c r="F11" s="162">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G11" s="160"/>
-      <c r="H11" s="159">
+      <c r="G11" s="163"/>
+      <c r="H11" s="162">
         <v>0.05</v>
       </c>
-      <c r="I11" s="160"/>
-      <c r="J11" s="159">
+      <c r="I11" s="163"/>
+      <c r="J11" s="162">
         <v>0.08</v>
       </c>
-      <c r="K11" s="160"/>
-      <c r="L11" s="159">
+      <c r="K11" s="163"/>
+      <c r="L11" s="162">
         <v>0.05</v>
       </c>
-      <c r="M11" s="160"/>
-      <c r="N11" s="159">
+      <c r="M11" s="163"/>
+      <c r="N11" s="162">
         <v>0.09</v>
       </c>
-      <c r="O11" s="160"/>
-      <c r="P11" s="159">
+      <c r="O11" s="163"/>
+      <c r="P11" s="162">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="Q11" s="160"/>
-      <c r="R11" s="159">
+      <c r="Q11" s="163"/>
+      <c r="R11" s="162">
         <v>0.04</v>
       </c>
-      <c r="S11" s="160"/>
-    </row>
-    <row r="12" spans="1:19" ht="17.100000000000001">
+      <c r="S11" s="163"/>
+    </row>
+    <row r="12" spans="1:19">
       <c r="A12" s="116" t="s">
         <v>288</v>
       </c>
-      <c r="B12" s="163">
+      <c r="B12" s="158">
         <v>713013</v>
       </c>
-      <c r="C12" s="163"/>
+      <c r="C12" s="158"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="52" t="s">
@@ -7677,6 +7677,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="R2:S2"/>
@@ -7693,7 +7694,6 @@
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7705,11 +7705,11 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:BU22"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="82.28515625" style="130" customWidth="1"/>
-    <col min="2" max="73" width="8.85546875" style="130" customWidth="1"/>
-    <col min="74" max="16384" width="10.85546875" style="130"/>
+    <col min="1" max="1" width="82.265625" style="130" customWidth="1"/>
+    <col min="2" max="73" width="8.86328125" style="130" customWidth="1"/>
+    <col min="74" max="16384" width="10.86328125" style="130"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:73" ht="198" customHeight="1">
@@ -7934,96 +7934,96 @@
       <c r="A2" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="161" t="s">
+      <c r="B2" s="159" t="s">
         <v>236</v>
       </c>
-      <c r="C2" s="162"/>
-      <c r="D2" s="162"/>
-      <c r="E2" s="162"/>
-      <c r="F2" s="162"/>
-      <c r="G2" s="162"/>
-      <c r="H2" s="162"/>
-      <c r="I2" s="162"/>
+      <c r="C2" s="160"/>
+      <c r="D2" s="160"/>
+      <c r="E2" s="160"/>
+      <c r="F2" s="160"/>
+      <c r="G2" s="160"/>
+      <c r="H2" s="160"/>
+      <c r="I2" s="160"/>
       <c r="J2" s="164"/>
-      <c r="K2" s="161" t="s">
+      <c r="K2" s="159" t="s">
         <v>238</v>
       </c>
-      <c r="L2" s="162"/>
-      <c r="M2" s="162"/>
-      <c r="N2" s="162"/>
-      <c r="O2" s="162"/>
-      <c r="P2" s="162"/>
-      <c r="Q2" s="162"/>
-      <c r="R2" s="162"/>
+      <c r="L2" s="160"/>
+      <c r="M2" s="160"/>
+      <c r="N2" s="160"/>
+      <c r="O2" s="160"/>
+      <c r="P2" s="160"/>
+      <c r="Q2" s="160"/>
+      <c r="R2" s="160"/>
       <c r="S2" s="164"/>
-      <c r="T2" s="161" t="s">
+      <c r="T2" s="159" t="s">
         <v>241</v>
       </c>
-      <c r="U2" s="162"/>
-      <c r="V2" s="162"/>
-      <c r="W2" s="162"/>
-      <c r="X2" s="162"/>
-      <c r="Y2" s="162"/>
-      <c r="Z2" s="162"/>
-      <c r="AA2" s="162"/>
+      <c r="U2" s="160"/>
+      <c r="V2" s="160"/>
+      <c r="W2" s="160"/>
+      <c r="X2" s="160"/>
+      <c r="Y2" s="160"/>
+      <c r="Z2" s="160"/>
+      <c r="AA2" s="160"/>
       <c r="AB2" s="164"/>
-      <c r="AC2" s="161" t="s">
+      <c r="AC2" s="159" t="s">
         <v>244</v>
       </c>
-      <c r="AD2" s="162"/>
-      <c r="AE2" s="162"/>
-      <c r="AF2" s="162"/>
-      <c r="AG2" s="162"/>
-      <c r="AH2" s="162"/>
-      <c r="AI2" s="162"/>
-      <c r="AJ2" s="162"/>
+      <c r="AD2" s="160"/>
+      <c r="AE2" s="160"/>
+      <c r="AF2" s="160"/>
+      <c r="AG2" s="160"/>
+      <c r="AH2" s="160"/>
+      <c r="AI2" s="160"/>
+      <c r="AJ2" s="160"/>
       <c r="AK2" s="164"/>
-      <c r="AL2" s="161" t="s">
+      <c r="AL2" s="159" t="s">
         <v>253</v>
       </c>
-      <c r="AM2" s="162"/>
-      <c r="AN2" s="162"/>
-      <c r="AO2" s="162"/>
-      <c r="AP2" s="162"/>
-      <c r="AQ2" s="162"/>
-      <c r="AR2" s="162"/>
-      <c r="AS2" s="162"/>
+      <c r="AM2" s="160"/>
+      <c r="AN2" s="160"/>
+      <c r="AO2" s="160"/>
+      <c r="AP2" s="160"/>
+      <c r="AQ2" s="160"/>
+      <c r="AR2" s="160"/>
+      <c r="AS2" s="160"/>
       <c r="AT2" s="164"/>
-      <c r="AU2" s="161" t="s">
+      <c r="AU2" s="159" t="s">
         <v>256</v>
       </c>
-      <c r="AV2" s="162"/>
-      <c r="AW2" s="162"/>
-      <c r="AX2" s="162"/>
-      <c r="AY2" s="162"/>
-      <c r="AZ2" s="162"/>
-      <c r="BA2" s="162"/>
-      <c r="BB2" s="162"/>
+      <c r="AV2" s="160"/>
+      <c r="AW2" s="160"/>
+      <c r="AX2" s="160"/>
+      <c r="AY2" s="160"/>
+      <c r="AZ2" s="160"/>
+      <c r="BA2" s="160"/>
+      <c r="BB2" s="160"/>
       <c r="BC2" s="164"/>
-      <c r="BD2" s="161" t="s">
+      <c r="BD2" s="159" t="s">
         <v>258</v>
       </c>
-      <c r="BE2" s="162"/>
-      <c r="BF2" s="162"/>
-      <c r="BG2" s="162"/>
-      <c r="BH2" s="162"/>
-      <c r="BI2" s="162"/>
-      <c r="BJ2" s="162"/>
-      <c r="BK2" s="162"/>
+      <c r="BE2" s="160"/>
+      <c r="BF2" s="160"/>
+      <c r="BG2" s="160"/>
+      <c r="BH2" s="160"/>
+      <c r="BI2" s="160"/>
+      <c r="BJ2" s="160"/>
+      <c r="BK2" s="160"/>
       <c r="BL2" s="164"/>
-      <c r="BM2" s="161" t="s">
+      <c r="BM2" s="159" t="s">
         <v>261</v>
       </c>
-      <c r="BN2" s="162"/>
-      <c r="BO2" s="162"/>
-      <c r="BP2" s="162"/>
-      <c r="BQ2" s="162"/>
-      <c r="BR2" s="162"/>
-      <c r="BS2" s="162"/>
-      <c r="BT2" s="162"/>
+      <c r="BN2" s="160"/>
+      <c r="BO2" s="160"/>
+      <c r="BP2" s="160"/>
+      <c r="BQ2" s="160"/>
+      <c r="BR2" s="160"/>
+      <c r="BS2" s="160"/>
+      <c r="BT2" s="160"/>
       <c r="BU2" s="164"/>
     </row>
-    <row r="3" spans="1:73" ht="17.100000000000001">
+    <row r="3" spans="1:73">
       <c r="A3" s="131" t="s">
         <v>298</v>
       </c>
@@ -8244,7 +8244,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:73" ht="17.100000000000001">
+    <row r="4" spans="1:73">
       <c r="A4" s="131" t="s">
         <v>299</v>
       </c>
@@ -8465,7 +8465,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:73" ht="17.100000000000001">
+    <row r="5" spans="1:73">
       <c r="A5" s="131" t="s">
         <v>300</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:73" ht="17.100000000000001">
+    <row r="6" spans="1:73">
       <c r="A6" s="131" t="s">
         <v>301</v>
       </c>
@@ -8907,7 +8907,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:73" ht="17.100000000000001">
+    <row r="7" spans="1:73">
       <c r="A7" s="131" t="s">
         <v>302</v>
       </c>
@@ -9128,7 +9128,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:73" ht="17.100000000000001">
+    <row r="8" spans="1:73">
       <c r="A8" s="131" t="s">
         <v>303</v>
       </c>
@@ -9349,7 +9349,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:73" ht="17.100000000000001">
+    <row r="9" spans="1:73">
       <c r="A9" s="131" t="s">
         <v>304</v>
       </c>
@@ -9570,7 +9570,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:73" ht="17.100000000000001">
+    <row r="10" spans="1:73">
       <c r="A10" s="131" t="s">
         <v>305</v>
       </c>
@@ -9791,7 +9791,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:73" ht="17.100000000000001">
+    <row r="11" spans="1:73">
       <c r="A11" s="131" t="s">
         <v>306</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="18.95">
+    <row r="22" spans="1:1" ht="18">
       <c r="A22" s="133"/>
     </row>
   </sheetData>
@@ -10041,11 +10041,11 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" style="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.85546875" style="36"/>
+    <col min="1" max="1" width="16.73046875" style="36" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.73046875" style="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.86328125" style="36"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -10227,13 +10227,13 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A2:H15"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" style="36" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="36"/>
-    <col min="3" max="3" width="14.42578125" style="36" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" style="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.85546875" style="36"/>
+    <col min="1" max="1" width="24.73046875" style="36" customWidth="1"/>
+    <col min="2" max="2" width="10.86328125" style="36"/>
+    <col min="3" max="3" width="14.3984375" style="36" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.265625" style="36" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.86328125" style="36"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="87" customHeight="1">
@@ -10532,20 +10532,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D29BF7EC-1543-BA40-9235-59CE5C807381}">
   <dimension ref="A1:U23"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="48.42578125" style="36" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="3" max="9" width="6.85546875" style="47" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" style="47" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="6.85546875" style="47" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="6.85546875" style="47" customWidth="1"/>
-    <col min="19" max="19" width="10.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.85546875" style="36" customWidth="1"/>
-    <col min="21" max="16384" width="8.85546875" style="36"/>
+    <col min="1" max="1" width="48.3984375" style="36" customWidth="1"/>
+    <col min="2" max="2" width="10.3984375" style="47" bestFit="1" customWidth="1"/>
+    <col min="3" max="9" width="6.86328125" style="47" customWidth="1"/>
+    <col min="10" max="10" width="10.3984375" style="47" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.86328125" style="47" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" style="47" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="6.86328125" style="47" customWidth="1"/>
+    <col min="15" max="15" width="10.3984375" style="47" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="6.86328125" style="47" customWidth="1"/>
+    <col min="19" max="19" width="10.3984375" style="47" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.86328125" style="36" customWidth="1"/>
+    <col min="21" max="16384" width="8.86328125" style="36"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="83.1" customHeight="1">
@@ -10607,7 +10607,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="89.1">
+    <row r="2" spans="1:21" ht="84.75">
       <c r="A2" s="43" t="s">
         <v>41</v>
       </c>
@@ -11563,7 +11563,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="U2">
-    <cfRule type="cellIs" dxfId="37" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11578,19 +11578,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E76B525B-8BE6-5E4E-9709-34D960252168}">
   <dimension ref="A2:AM90"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="51" style="36" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="47"/>
-    <col min="3" max="3" width="13.42578125" style="47" customWidth="1"/>
-    <col min="4" max="16384" width="10.85546875" style="36"/>
+    <col min="2" max="2" width="10.86328125" style="47"/>
+    <col min="3" max="3" width="13.3984375" style="47" customWidth="1"/>
+    <col min="4" max="16384" width="10.86328125" style="36"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:39" ht="113.1">
-      <c r="B2" s="150" t="s">
+    <row r="2" spans="1:39" ht="112.15">
+      <c r="B2" s="152" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="150" t="s">
+      <c r="C2" s="152" t="s">
         <v>59</v>
       </c>
       <c r="D2" s="54" t="s">
@@ -11706,8 +11706,8 @@
       <c r="A3" s="53" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="151"/>
-      <c r="C3" s="151"/>
+      <c r="B3" s="153"/>
+      <c r="C3" s="153"/>
       <c r="D3" s="148" t="s">
         <v>3</v>
       </c>
@@ -11720,10 +11720,10 @@
         <v>7</v>
       </c>
       <c r="I3" s="149"/>
-      <c r="J3" s="152" t="s">
+      <c r="J3" s="154" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="153"/>
+      <c r="K3" s="155"/>
       <c r="L3" s="148" t="s">
         <v>12</v>
       </c>
@@ -11740,10 +11740,10 @@
         <v>18</v>
       </c>
       <c r="S3" s="149"/>
-      <c r="T3" s="154" t="s">
+      <c r="T3" s="156" t="s">
         <v>20</v>
       </c>
-      <c r="U3" s="155"/>
+      <c r="U3" s="157"/>
       <c r="V3" s="148" t="s">
         <v>22</v>
       </c>
@@ -11760,10 +11760,10 @@
         <v>28</v>
       </c>
       <c r="AC3" s="149"/>
-      <c r="AD3" s="156" t="s">
+      <c r="AD3" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="157"/>
+      <c r="AE3" s="151"/>
       <c r="AF3" s="148" t="s">
         <v>26</v>
       </c>
@@ -11781,7 +11781,7 @@
       </c>
       <c r="AM3" s="149"/>
     </row>
-    <row r="4" spans="1:39" ht="33.950000000000003">
+    <row r="4" spans="1:39" ht="31.5">
       <c r="A4" s="57" t="s">
         <v>97</v>
       </c>
@@ -11846,7 +11846,7 @@
       <c r="AL4" s="49"/>
       <c r="AM4" s="49"/>
     </row>
-    <row r="5" spans="1:39" ht="33.950000000000003">
+    <row r="5" spans="1:39" ht="31.5">
       <c r="A5" s="57" t="s">
         <v>98</v>
       </c>
@@ -11911,7 +11911,7 @@
       <c r="AL5" s="49"/>
       <c r="AM5" s="49"/>
     </row>
-    <row r="6" spans="1:39" ht="33.950000000000003">
+    <row r="6" spans="1:39" ht="31.5">
       <c r="A6" s="57" t="s">
         <v>99</v>
       </c>
@@ -11976,7 +11976,7 @@
       <c r="AL6" s="49"/>
       <c r="AM6" s="49"/>
     </row>
-    <row r="7" spans="1:39" ht="17.100000000000001">
+    <row r="7" spans="1:39" ht="31.5">
       <c r="A7" s="57" t="s">
         <v>100</v>
       </c>
@@ -12041,7 +12041,7 @@
       <c r="AL7" s="49"/>
       <c r="AM7" s="49"/>
     </row>
-    <row r="8" spans="1:39" ht="33.950000000000003">
+    <row r="8" spans="1:39" ht="31.5">
       <c r="A8" s="57" t="s">
         <v>101</v>
       </c>
@@ -12106,7 +12106,7 @@
       <c r="AL8" s="49"/>
       <c r="AM8" s="49"/>
     </row>
-    <row r="9" spans="1:39" ht="33.950000000000003">
+    <row r="9" spans="1:39" ht="31.5">
       <c r="A9" s="57" t="s">
         <v>102</v>
       </c>
@@ -12171,7 +12171,7 @@
       <c r="AL9" s="49"/>
       <c r="AM9" s="49"/>
     </row>
-    <row r="10" spans="1:39" ht="33.950000000000003">
+    <row r="10" spans="1:39" ht="31.5">
       <c r="A10" s="57" t="s">
         <v>103</v>
       </c>
@@ -12236,7 +12236,7 @@
       <c r="AL10" s="49"/>
       <c r="AM10" s="49"/>
     </row>
-    <row r="11" spans="1:39" ht="33.950000000000003">
+    <row r="11" spans="1:39" ht="31.5">
       <c r="A11" s="57" t="s">
         <v>104</v>
       </c>
@@ -12301,7 +12301,7 @@
       <c r="AL11" s="49"/>
       <c r="AM11" s="49"/>
     </row>
-    <row r="12" spans="1:39" ht="33.950000000000003">
+    <row r="12" spans="1:39" ht="31.5">
       <c r="A12" s="57" t="s">
         <v>105</v>
       </c>
@@ -12366,7 +12366,7 @@
       <c r="AL12" s="49"/>
       <c r="AM12" s="49"/>
     </row>
-    <row r="13" spans="1:39" ht="33.950000000000003">
+    <row r="13" spans="1:39" ht="31.5">
       <c r="A13" s="57" t="s">
         <v>106</v>
       </c>
@@ -12419,7 +12419,7 @@
       <c r="AL13" s="49"/>
       <c r="AM13" s="49"/>
     </row>
-    <row r="14" spans="1:39" ht="17.100000000000001">
+    <row r="14" spans="1:39">
       <c r="A14" s="57" t="s">
         <v>107</v>
       </c>
@@ -12489,7 +12489,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="79" spans="1:21" ht="18.95">
+    <row r="79" spans="1:21" ht="18">
       <c r="A79" s="53" t="s">
         <v>96</v>
       </c>
@@ -12913,14 +12913,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="AJ3:AK3"/>
-    <mergeCell ref="AL3:AM3"/>
-    <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="AH3:AI3"/>
     <mergeCell ref="V3:W3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
@@ -12933,6 +12925,14 @@
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="R3:S3"/>
     <mergeCell ref="T3:U3"/>
+    <mergeCell ref="AJ3:AK3"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="AB3:AC3"/>
+    <mergeCell ref="AD3:AE3"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="AH3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12945,16 +12945,16 @@
     <tabColor theme="7" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="63" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="15.73046875" style="63" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="49" style="63" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="0" style="62" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="41.7109375" style="62" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="41.73046875" style="62" hidden="1" customWidth="1"/>
     <col min="5" max="8" width="0" style="62" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" style="72" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="46.7109375" style="72" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.85546875" style="62"/>
+    <col min="9" max="9" width="19.73046875" style="72" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="46.73046875" style="72" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.86328125" style="62"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -13384,17 +13384,17 @@
     <tabColor theme="7" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:N15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="11.1"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="10.5"/>
   <cols>
     <col min="1" max="1" width="32" style="91" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="80" customWidth="1"/>
+    <col min="2" max="2" width="6.265625" style="80" customWidth="1"/>
     <col min="3" max="3" width="7" style="80" customWidth="1"/>
-    <col min="4" max="10" width="6.28515625" style="80" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="80"/>
-    <col min="12" max="12" width="9.28515625" style="80" bestFit="1" customWidth="1"/>
+    <col min="4" max="10" width="6.265625" style="80" customWidth="1"/>
+    <col min="11" max="11" width="9.1328125" style="80"/>
+    <col min="12" max="12" width="9.265625" style="80" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" style="80" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" style="80" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="80"/>
+    <col min="14" max="14" width="9.265625" style="80" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.1328125" style="80"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="105.95" customHeight="1">
@@ -13695,7 +13695,7 @@
       </c>
       <c r="K9" s="79"/>
     </row>
-    <row r="15" spans="1:14" ht="15.95">
+    <row r="15" spans="1:14" ht="15.75">
       <c r="A15" s="92" t="s">
         <v>187</v>
       </c>
@@ -13740,17 +13740,17 @@
     <tabColor theme="7" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Q17"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="11.1"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="10.5"/>
   <cols>
     <col min="1" max="1" width="32" style="91" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="80" customWidth="1"/>
+    <col min="2" max="2" width="6.265625" style="80" customWidth="1"/>
     <col min="3" max="3" width="7" style="80" customWidth="1"/>
-    <col min="4" max="10" width="6.28515625" style="80" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="80"/>
-    <col min="12" max="12" width="9.28515625" style="80" bestFit="1" customWidth="1"/>
+    <col min="4" max="10" width="6.265625" style="80" customWidth="1"/>
+    <col min="11" max="11" width="9.1328125" style="80"/>
+    <col min="12" max="12" width="9.265625" style="80" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" style="80" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" style="80" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="80"/>
+    <col min="14" max="14" width="9.265625" style="80" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.1328125" style="80"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75" customHeight="1">
@@ -14047,7 +14047,7 @@
       <c r="M11" s="102"/>
       <c r="N11" s="103"/>
     </row>
-    <row r="17" spans="1:1" ht="15.95">
+    <row r="17" spans="1:1" ht="15.75">
       <c r="A17" s="92" t="s">
         <v>187</v>
       </c>
@@ -14068,15 +14068,15 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:D40"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="13.15"/>
   <cols>
     <col min="1" max="1" width="19" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="10.85546875" style="2"/>
+    <col min="2" max="2" width="22.86328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.3984375" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="10.86328125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="15.75">
       <c r="A1" s="4" t="s">
         <v>192</v>
       </c>
@@ -14105,7 +14105,7 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="1:4" ht="17.100000000000001">
+    <row r="4" spans="1:4" ht="15.75">
       <c r="A4" s="5" t="s">
         <v>198</v>
       </c>
@@ -14115,7 +14115,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4" ht="17.100000000000001">
+    <row r="5" spans="1:4" ht="15.75">
       <c r="A5" s="5" t="s">
         <v>200</v>
       </c>
@@ -14125,7 +14125,7 @@
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:4" ht="17.100000000000001">
+    <row r="6" spans="1:4" ht="31.5">
       <c r="A6" s="5" t="s">
         <v>202</v>
       </c>
@@ -14135,7 +14135,7 @@
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4" ht="17.100000000000001">
+    <row r="7" spans="1:4" ht="31.5">
       <c r="A7" s="5" t="s">
         <v>204</v>
       </c>
@@ -14145,7 +14145,7 @@
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4" ht="17.100000000000001">
+    <row r="8" spans="1:4" ht="15.75">
       <c r="A8" s="5" t="s">
         <v>205</v>
       </c>
@@ -14155,7 +14155,7 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4" ht="17.100000000000001">
+    <row r="9" spans="1:4" ht="15.75">
       <c r="A9" s="5" t="s">
         <v>207</v>
       </c>
@@ -14165,7 +14165,7 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4" ht="17.100000000000001">
+    <row r="10" spans="1:4" ht="15.75">
       <c r="A10" s="5" t="s">
         <v>208</v>
       </c>
@@ -14175,7 +14175,7 @@
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
     </row>
-    <row r="11" spans="1:4" ht="17.100000000000001">
+    <row r="11" spans="1:4" ht="15.75">
       <c r="A11" s="5" t="s">
         <v>210</v>
       </c>
@@ -14185,7 +14185,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
     </row>
-    <row r="12" spans="1:4" ht="17.100000000000001">
+    <row r="12" spans="1:4" ht="15.75">
       <c r="A12" s="5" t="s">
         <v>211</v>
       </c>
@@ -14195,7 +14195,7 @@
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4" ht="17.100000000000001">
+    <row r="13" spans="1:4" ht="15.75">
       <c r="A13" s="5" t="s">
         <v>212</v>
       </c>
@@ -14205,7 +14205,7 @@
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
     </row>
-    <row r="14" spans="1:4" ht="17.100000000000001">
+    <row r="14" spans="1:4" ht="15.75">
       <c r="A14" s="5" t="s">
         <v>214</v>
       </c>
@@ -14215,7 +14215,7 @@
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
     </row>
-    <row r="15" spans="1:4" ht="17.100000000000001">
+    <row r="15" spans="1:4" ht="15.75">
       <c r="A15" s="5" t="s">
         <v>215</v>
       </c>
@@ -14225,7 +14225,7 @@
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
     </row>
-    <row r="16" spans="1:4" ht="17.100000000000001">
+    <row r="16" spans="1:4" ht="15.75">
       <c r="A16" s="5" t="s">
         <v>217</v>
       </c>
@@ -14235,7 +14235,7 @@
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
     </row>
-    <row r="17" spans="1:4" ht="17.100000000000001">
+    <row r="17" spans="1:4" ht="15.75">
       <c r="A17" s="5" t="s">
         <v>219</v>
       </c>
@@ -14245,7 +14245,7 @@
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
     </row>
-    <row r="18" spans="1:4" ht="17.100000000000001">
+    <row r="18" spans="1:4" ht="15.75">
       <c r="A18" s="5" t="s">
         <v>221</v>
       </c>
@@ -14255,7 +14255,7 @@
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="1:4" ht="17.100000000000001">
+    <row r="19" spans="1:4" ht="15.75">
       <c r="A19" s="5" t="s">
         <v>222</v>
       </c>
@@ -14265,7 +14265,7 @@
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
     </row>
-    <row r="20" spans="1:4" ht="17.100000000000001">
+    <row r="20" spans="1:4" ht="15.75">
       <c r="A20" s="5" t="s">
         <v>223</v>
       </c>
@@ -14275,7 +14275,7 @@
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
     </row>
-    <row r="21" spans="1:4" ht="17.100000000000001">
+    <row r="21" spans="1:4" ht="15.75">
       <c r="A21" s="5" t="s">
         <v>224</v>
       </c>
@@ -14285,115 +14285,115 @@
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
     </row>
-    <row r="22" spans="1:4" ht="15.95">
+    <row r="22" spans="1:4" ht="15.75">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
     </row>
-    <row r="23" spans="1:4" ht="15.95">
+    <row r="23" spans="1:4" ht="15.75">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
     </row>
-    <row r="24" spans="1:4" ht="15.95">
+    <row r="24" spans="1:4" ht="15.75">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
     </row>
-    <row r="25" spans="1:4" ht="15.95">
+    <row r="25" spans="1:4" ht="15.75">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="1:4" ht="15.95">
+    <row r="26" spans="1:4" ht="15.75">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
     </row>
-    <row r="27" spans="1:4" ht="15.95">
+    <row r="27" spans="1:4" ht="15.75">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
     </row>
-    <row r="28" spans="1:4" ht="15.95">
+    <row r="28" spans="1:4" ht="15.75">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
     </row>
-    <row r="29" spans="1:4" ht="15.95">
+    <row r="29" spans="1:4" ht="15.75">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
     </row>
-    <row r="30" spans="1:4" ht="15.95">
+    <row r="30" spans="1:4" ht="15.75">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
     </row>
-    <row r="31" spans="1:4" ht="15.95">
+    <row r="31" spans="1:4" ht="15.75">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
     </row>
-    <row r="32" spans="1:4" ht="15.95">
+    <row r="32" spans="1:4" ht="15.75">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
     </row>
-    <row r="33" spans="1:4" ht="15.95">
+    <row r="33" spans="1:4" ht="15.75">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
     </row>
-    <row r="34" spans="1:4" ht="15.95">
+    <row r="34" spans="1:4" ht="15.75">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
     </row>
-    <row r="35" spans="1:4" ht="15.95">
+    <row r="35" spans="1:4" ht="15.75">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
     </row>
-    <row r="36" spans="1:4" ht="15.95">
+    <row r="36" spans="1:4" ht="15.75">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
-    <row r="37" spans="1:4" ht="15.95">
+    <row r="37" spans="1:4" ht="15.75">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
     </row>
-    <row r="38" spans="1:4" ht="15.95">
+    <row r="38" spans="1:4" ht="15.75">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
     </row>
-    <row r="39" spans="1:4" ht="15.95">
+    <row r="39" spans="1:4" ht="15.75">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
-    <row r="40" spans="1:4" ht="15.95">
+    <row r="40" spans="1:4" ht="15.75">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -14410,19 +14410,19 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A2:L17"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="13.15"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.19921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="7.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.265625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="10.85546875" style="1"/>
+    <col min="12" max="16384" width="10.86328125" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="69.95" customHeight="1">
@@ -14493,7 +14493,7 @@
       </c>
       <c r="L3" s="17"/>
     </row>
-    <row r="4" spans="1:12" ht="51">
+    <row r="4" spans="1:12" ht="47.25">
       <c r="A4" s="20" t="s">
         <v>230</v>
       </c>
@@ -14532,7 +14532,7 @@
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
     </row>
-    <row r="6" spans="1:12" ht="17.100000000000001">
+    <row r="6" spans="1:12" ht="15.75">
       <c r="A6" s="20" t="s">
         <v>231</v>
       </c>
@@ -14563,7 +14563,7 @@
         <v>311210</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="51">
+    <row r="9" spans="1:12" ht="47.25">
       <c r="A9" s="20" t="s">
         <v>232</v>
       </c>
@@ -14596,7 +14596,7 @@
         <v>9636.5798014202628</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15.95">
+    <row r="17" spans="1:1" ht="15.75">
       <c r="A17" s="19" t="s">
         <v>108</v>
       </c>
@@ -14612,11 +14612,11 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="16" style="36" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" style="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.85546875" style="36"/>
+    <col min="3" max="16384" width="10.86328125" style="36"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -14793,6 +14793,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010058F4C97533AB4D4AB0E3CF7046F02B9B" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cd3ec89b4fa8ac99d6316b2e27026dd1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aec805b8-e1f0-47ef-9b62-e279cd33bd3b" xmlns:ns3="623b8ea9-3cd3-401a-a35a-6ba6e3f85b77" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="497fc33add14695dc9b4e6c3722c7d90" ns2:_="" ns3:_="">
     <xsd:import namespace="aec805b8-e1f0-47ef-9b62-e279cd33bd3b"/>
@@ -15033,15 +15042,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -15054,13 +15054,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04349A01-CB34-49EE-94A6-60078C44FB89}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADDD680D-6999-4ED0-B19D-4BCDB9388D45}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADDD680D-6999-4ED0-B19D-4BCDB9388D45}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04349A01-CB34-49EE-94A6-60078C44FB89}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="aec805b8-e1f0-47ef-9b62-e279cd33bd3b"/>
+    <ds:schemaRef ds:uri="623b8ea9-3cd3-401a-a35a-6ba6e3f85b77"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A81FF801-A863-463E-9912-37F7E378BE07}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A81FF801-A863-463E-9912-37F7E378BE07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="aec805b8-e1f0-47ef-9b62-e279cd33bd3b"/>
+    <ds:schemaRef ds:uri="623b8ea9-3cd3-401a-a35a-6ba6e3f85b77"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>